<commit_message>
base base case model
</commit_message>
<xml_diff>
--- a/Docs/Thesis planning.xlsx
+++ b/Docs/Thesis planning.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/LaptopvanFrank/Desktop/Cardano/Thesis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C8BC523-A733-834F-A891-FDB254883468}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{286A0EFA-9132-8348-9033-45B65205F6B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20460" xr2:uid="{C4A47A45-E97D-B144-962D-ED697A072EEA}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="34560" windowHeight="21600" xr2:uid="{C4A47A45-E97D-B144-962D-ED697A072EEA}"/>
   </bookViews>
   <sheets>
     <sheet name="-" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="43">
   <si>
     <t xml:space="preserve">Thesis planning </t>
   </si>
@@ -47,9 +47,6 @@
     <t>Subject</t>
   </si>
   <si>
-    <t>Uni supervisor</t>
-  </si>
-  <si>
     <t>Company supervisor</t>
   </si>
   <si>
@@ -71,9 +68,6 @@
     <t>Roel Mehlkopf</t>
   </si>
   <si>
-    <t>Optimization and hedging of liability-driven investment portfolios under Wtp: earning the protection return</t>
-  </si>
-  <si>
     <t>Start date</t>
   </si>
   <si>
@@ -84,9 +78,6 @@
   </si>
   <si>
     <t>Achieved</t>
-  </si>
-  <si>
-    <t>Deadline passed</t>
   </si>
   <si>
     <t>ma, wo, do: Collateral
@@ -96,26 +87,6 @@
     <t>Papers Lezen + Base Case model</t>
   </si>
   <si>
-    <t>Base Case Model</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">ma, wo, do: Collateral
-di, vr: Thesis
-</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>8 okt 10.00 JvL</t>
-    </r>
-  </si>
-  <si>
     <t>Brainstorming onderzoeksrichting, proposal opstellen</t>
   </si>
   <si>
@@ -144,12 +115,6 @@
     <t>Onderzoeksresulaten</t>
   </si>
   <si>
-    <t>Papers Lezen</t>
-  </si>
-  <si>
-    <t>Probleemomschrijving</t>
-  </si>
-  <si>
     <t>Introductie</t>
   </si>
   <si>
@@ -165,20 +130,55 @@
     <t>Plan van aanpak</t>
   </si>
   <si>
-    <t>Model finalizeren</t>
-  </si>
-  <si>
     <t>Inleveren verslag</t>
   </si>
   <si>
     <t>Resultaten + Verslag</t>
+  </si>
+  <si>
+    <t>Probleemomschrijving + Model Formulation Final</t>
+  </si>
+  <si>
+    <t>Probleemomschrijving + Model Formulation Proposal</t>
+  </si>
+  <si>
+    <t>D-day: Thesis verdediging</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Model </t>
+  </si>
+  <si>
+    <t>Snowboarden</t>
+  </si>
+  <si>
+    <t>Optimization and hedging of liability-driven investment portfolios under Wtp: extending the Merton model with mismatch risk</t>
+  </si>
+  <si>
+    <t>Deadline passed/
+Absent</t>
+  </si>
+  <si>
+    <t>University supervisor</t>
+  </si>
+  <si>
+    <t>wo, do, vr: Collateral 
+ma, di: Thesis</t>
+  </si>
+  <si>
+    <t>Wintersport - Hintertux/Tux</t>
+  </si>
+  <si>
+    <t>Papers Lezen + Base Case model + Model bouwen</t>
+  </si>
+  <si>
+    <t>Base case model script + progressie PP</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -231,14 +231,30 @@
     <font>
       <i/>
       <sz val="12"/>
+      <color rgb="FF9C0006"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <strike/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <strike/>
+      <sz val="12"/>
       <color rgb="FF006100"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
     <font>
       <i/>
+      <strike/>
       <sz val="12"/>
-      <color rgb="FF9C0006"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
@@ -266,7 +282,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -304,37 +320,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -396,6 +381,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -403,7 +408,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -416,22 +421,31 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="10" xfId="3" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="7" xfId="3" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Bad" xfId="2" builtinId="27"/>
@@ -450,6 +464,259 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="TextBox 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1D8A604C-6D88-9231-E961-C5B3916A75EE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="12077700" y="3479800"/>
+          <a:ext cx="3098800" cy="1663700"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="25400" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="tx1"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100" b="1"/>
+            <a:t>Structuur verslag:</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100"/>
+            <a:t>	1. Intro</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100"/>
+            <a:t>	2. Probleemomschrijving</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100"/>
+            <a:t>	3. Literatuurstudie</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100"/>
+            <a:t>	4. Plan van aanpak</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100"/>
+            <a:t>	5. Model</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100"/>
+            <a:t>	6. Onderzoeksresultaten</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100"/>
+            <a:t>	7. Conclusie &amp; Aanbevelingen</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100"/>
+            <a:t>	8. Appendix</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>698500</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>366598</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="TextBox 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F81E24F6-3F98-B24E-8A69-72979B1F49F7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="12071546" y="5729926"/>
+          <a:ext cx="8698191" cy="1942445"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="25400" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="tx1"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100" b="1"/>
+            <a:t>Papers:</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr rtl="0"/>
+          <a:r>
+            <a:rPr lang="en-NL"/>
+            <a:t>	1. Lifetime Portfolio Selection under Uncertainty: The Continuous-Time Case, Merton, 1969</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr rtl="0"/>
+          <a:r>
+            <a:rPr lang="en-NL"/>
+            <a:t>	2. Liabilities – A New Approach, Sharpe &amp; Tint, 1990</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr rtl="0"/>
+          <a:r>
+            <a:rPr lang="en-NL"/>
+            <a:t>	3. Optimal Design of Funded Pension Schemes, Bovenberg &amp; Mehlkopf, 2014</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr rtl="0"/>
+          <a:r>
+            <a:rPr lang="en-NL"/>
+            <a:t>	4. Is er nog ruimte voor obligaties binnen de beschermingsportefeuille?, Ernsting et al., 2025</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr rtl="0"/>
+          <a:r>
+            <a:rPr lang="en-NL"/>
+            <a:t>	5. Beschermings-, over- en projectierendementen, Werker, 2022</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr rtl="0"/>
+          <a:r>
+            <a:rPr lang="en-NL"/>
+            <a:t>	6. Beschermingsrendement: Theoretisch of praktisch?, Potter van Loon &amp; Alserda, 2025</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr rtl="0"/>
+          <a:r>
+            <a:rPr lang="en-NL"/>
+            <a:t>	7.</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-NL" baseline="0"/>
+            <a:t> </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-NL"/>
+            <a:t>Renterisico, lifecycle en pensioencontract, Mehlkopf &amp; Van Bilsen, 2020</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr rtl="0"/>
+          <a:r>
+            <a:rPr lang="en-NL"/>
+            <a:t>	8. </a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -769,7 +1036,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98254ADD-4174-6640-B5B6-8A09C76A8B6C}">
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
@@ -777,442 +1044,482 @@
     <col min="3" max="3" width="54.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="43.5" customWidth="1"/>
     <col min="5" max="5" width="15.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
     </row>
-    <row r="2" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" s="11" t="s">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" s="17" t="s">
+      <c r="A3" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
-        <v>22</v>
-      </c>
-      <c r="F3" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="G3" s="19"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" s="17" t="s">
-        <v>3</v>
-      </c>
       <c r="B4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" s="11" t="s">
         <v>9</v>
-      </c>
-      <c r="F4" s="20" t="s">
-        <v>13</v>
-      </c>
-      <c r="G4" s="21"/>
-    </row>
-    <row r="5" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="17" t="s">
-        <v>11</v>
       </c>
       <c r="B5" s="5">
         <v>46288</v>
       </c>
-      <c r="F5" s="22" t="s">
-        <v>14</v>
-      </c>
-      <c r="G5" s="23"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A6" s="17" t="s">
-        <v>12</v>
+      <c r="A6" s="11" t="s">
+        <v>10</v>
       </c>
       <c r="B6" s="5">
         <v>46500</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="C8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="D8" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D8" s="1" t="s">
+    </row>
+    <row r="9" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+      <c r="A9" s="21" t="str">
+        <f>"Week "&amp;_xlfn.LET(_xlpm.d,"21-9-2026"+7*(ROWS($A$1:A1)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
+        <v>Week 39: 21 Sep-25 Sep</v>
+      </c>
+      <c r="B9" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="23" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" s="24" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A9" s="3" t="str">
-        <f ca="1">"Week "&amp;_xlfn.LET(_xlpm.d,TODAY()+7*(ROWS($A$1:A1)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
-        <v>Week 39: 21 Sep-25 Sep</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="C9" t="s">
-        <v>20</v>
-      </c>
-      <c r="D9" s="14" t="s">
-        <v>8</v>
-      </c>
+      <c r="F9" s="26" t="s">
+        <v>37</v>
+      </c>
+      <c r="G9" s="12"/>
     </row>
     <row r="10" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A10" s="3" t="str">
-        <f ca="1">"Week "&amp;_xlfn.LET(_xlpm.d,TODAY()+7*(ROWS($A$1:A2)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
+      <c r="A10" s="21" t="str">
+        <f>"Week "&amp;_xlfn.LET(_xlpm.d,"21-9-2026"+7*(ROWS($A$1:A2)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
         <v>Week 40: 28 Sep-2 Oct</v>
       </c>
-      <c r="B10" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="C10" t="s">
-        <v>17</v>
-      </c>
-      <c r="D10" s="4"/>
-    </row>
-    <row r="11" spans="1:7" ht="51" x14ac:dyDescent="0.2">
-      <c r="A11" s="3" t="str">
-        <f ca="1">"Week "&amp;_xlfn.LET(_xlpm.d,TODAY()+7*(ROWS($A$1:A3)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
+      <c r="B10" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10" s="25"/>
+      <c r="F10" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="G10" s="14"/>
+    </row>
+    <row r="11" spans="1:7" ht="35" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="21" t="str">
+        <f>"Week "&amp;_xlfn.LET(_xlpm.d,"21-9-2026"+7*(ROWS($A$1:A3)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
         <v>Week 41: 5 Oct-9 Oct</v>
       </c>
-      <c r="B11" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="C11" t="s">
-        <v>17</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>18</v>
-      </c>
+      <c r="B11" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="D11" s="24" t="s">
+        <v>32</v>
+      </c>
+      <c r="F11" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="G11" s="16"/>
     </row>
     <row r="12" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A12" s="3" t="str">
-        <f ca="1">"Week "&amp;_xlfn.LET(_xlpm.d,TODAY()+7*(ROWS($A$1:A4)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
+      <c r="A12" s="21" t="str">
+        <f>"Week "&amp;_xlfn.LET(_xlpm.d,"21-9-2026"+7*(ROWS($A$1:A4)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
         <v>Week 42: 12 Oct-16 Oct</v>
       </c>
-      <c r="B12" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="C12" t="s">
-        <v>29</v>
+      <c r="B12" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="C12" s="23" t="s">
+        <v>14</v>
       </c>
       <c r="D12" s="4"/>
     </row>
     <row r="13" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="str">
-        <f ca="1">"Week "&amp;_xlfn.LET(_xlpm.d,TODAY()+7*(ROWS($A$1:A5)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
+        <f>"Week "&amp;_xlfn.LET(_xlpm.d,"21-9-2026"+7*(ROWS($A$1:A5)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
         <v>Week 43: 19 Oct-23 Oct</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="C13" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>30</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="F13" s="7"/>
     </row>
     <row r="14" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="str">
-        <f ca="1">"Week "&amp;_xlfn.LET(_xlpm.d,TODAY()+7*(ROWS($A$1:A6)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
+        <f>"Week "&amp;_xlfn.LET(_xlpm.d,"21-9-2026"+7*(ROWS($A$1:A6)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
         <v>Week 44: 26 Oct-30 Oct</v>
       </c>
       <c r="B14" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C14" t="s">
         <v>26</v>
       </c>
-      <c r="C14" t="s">
-        <v>33</v>
-      </c>
-      <c r="D14" s="4"/>
+      <c r="D14" s="4" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="15" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="str">
-        <f ca="1">"Week "&amp;_xlfn.LET(_xlpm.d,TODAY()+7*(ROWS($A$1:A7)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
+        <f>"Week "&amp;_xlfn.LET(_xlpm.d,"21-9-2026"+7*(ROWS($A$1:A7)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
         <v>Week 45: 2 Nov-6 Nov</v>
       </c>
       <c r="B15" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C15" t="s">
         <v>26</v>
-      </c>
-      <c r="C15" t="s">
-        <v>33</v>
       </c>
       <c r="D15" s="4"/>
     </row>
     <row r="16" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="str">
-        <f ca="1">"Week "&amp;_xlfn.LET(_xlpm.d,TODAY()+7*(ROWS($A$1:A8)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
+        <f>"Week "&amp;_xlfn.LET(_xlpm.d,"21-9-2026"+7*(ROWS($A$1:A8)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
         <v>Week 46: 9 Nov-13 Nov</v>
       </c>
       <c r="B16" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C16" t="s">
         <v>26</v>
       </c>
-      <c r="C16" t="s">
-        <v>33</v>
-      </c>
       <c r="D16" s="4" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="str">
-        <f ca="1">"Week "&amp;_xlfn.LET(_xlpm.d,TODAY()+7*(ROWS($A$1:A9)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
+        <f>"Week "&amp;_xlfn.LET(_xlpm.d,"21-9-2026"+7*(ROWS($A$1:A9)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
         <v>Week 47: 16 Nov-20 Nov</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C17" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="D17" s="4"/>
     </row>
     <row r="18" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A18" s="3" t="str">
-        <f ca="1">"Week "&amp;_xlfn.LET(_xlpm.d,TODAY()+7*(ROWS($A$1:A10)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
+        <f>"Week "&amp;_xlfn.LET(_xlpm.d,"21-9-2026"+7*(ROWS($A$1:A10)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
         <v>Week 48: 23 Nov-27 Nov</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C18" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="D18" s="4"/>
     </row>
     <row r="19" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="str">
-        <f ca="1">"Week "&amp;_xlfn.LET(_xlpm.d,TODAY()+7*(ROWS($A$1:A11)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
+        <f>"Week "&amp;_xlfn.LET(_xlpm.d,"21-9-2026"+7*(ROWS($A$1:A11)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
         <v>Week 49: 30 Nov-4 Dec</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C19" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="str">
-        <f ca="1">"Week "&amp;_xlfn.LET(_xlpm.d,TODAY()+7*(ROWS($A$1:A12)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
+        <f>"Week "&amp;_xlfn.LET(_xlpm.d,"21-9-2026"+7*(ROWS($A$1:A12)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
         <v>Week 50: 7 Dec-11 Dec</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C20" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="D20" s="4"/>
     </row>
     <row r="21" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="str">
-        <f ca="1">"Week "&amp;_xlfn.LET(_xlpm.d,TODAY()+7*(ROWS($A$1:A15)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
-        <v>Week 53: 28 Dec-1 Jan</v>
+        <f>"Week "&amp;_xlfn.LET(_xlpm.d,"21-9-2026"+7*(ROWS($A$1:A13)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
+        <v>Week 51: 14 Dec-18 Dec</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C21" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="D21" s="4"/>
     </row>
     <row r="22" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="str">
-        <f ca="1">"Week "&amp;_xlfn.LET(_xlpm.d,TODAY()+7*(ROWS($A$1:A16)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
-        <v>Week 1: 4 Jan-8 Jan</v>
+        <f>"Week "&amp;_xlfn.LET(_xlpm.d,"21-9-2026"+7*(ROWS($A$1:A14)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
+        <v>Week 52: 21 Dec-25 Dec</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C22" t="s">
-        <v>34</v>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" s="8" t="str">
-        <f ca="1">"Week "&amp;_xlfn.LET(_xlpm.d,TODAY()+7*(ROWS($A$1:A17)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
-        <v>Week 2: 11 Jan-15 Jan</v>
-      </c>
-      <c r="B23" s="6"/>
+      <c r="A23" s="3" t="str">
+        <f>"Week "&amp;_xlfn.LET(_xlpm.d,"21-9-2026"+7*(ROWS($A$1:A15)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
+        <v>Week 53: 28 Dec-1 Jan</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="C23" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="D23" s="15" t="s">
-        <v>25</v>
+        <v>19</v>
+      </c>
+      <c r="D23" s="9" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="str">
-        <f ca="1">"Week "&amp;_xlfn.LET(_xlpm.d,TODAY()+7*(ROWS($A$1:A18)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
-        <v>Week 3: 18 Jan-22 Jan</v>
+        <f>"Week "&amp;_xlfn.LET(_xlpm.d,"21-9-2026"+7*(ROWS($A$1:A16)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
+        <v>Week 1: 4 Jan-8 Jan</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C24" t="s">
-        <v>38</v>
-      </c>
-      <c r="D24" s="4"/>
+        <v>27</v>
+      </c>
     </row>
     <row r="25" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A25" s="3" t="str">
-        <f ca="1">"Week "&amp;_xlfn.LET(_xlpm.d,TODAY()+7*(ROWS($A$1:A19)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
-        <v>Week 4: 25 Jan-29 Jan</v>
+        <f>"Week "&amp;_xlfn.LET(_xlpm.d,"21-9-2026"+7*(ROWS($A$1:A17)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
+        <v>Week 2: 11 Jan-15 Jan</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C25" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="str">
-        <f ca="1">"Week "&amp;_xlfn.LET(_xlpm.d,TODAY()+7*(ROWS($A$1:A20)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
-        <v>Week 5: 1 Feb-5 Feb</v>
+        <f>"Week "&amp;_xlfn.LET(_xlpm.d,"21-9-2026"+7*(ROWS($A$1:A18)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
+        <v>Week 3: 18 Jan-22 Jan</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C26" t="s">
-        <v>23</v>
-      </c>
-      <c r="D26" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A27" s="3" t="str">
-        <f ca="1">"Week "&amp;_xlfn.LET(_xlpm.d,TODAY()+7*(ROWS($A$1:A21)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
-        <v>Week 6: 8 Feb-12 Feb</v>
+        <f>"Week "&amp;_xlfn.LET(_xlpm.d,"21-9-2026"+7*(ROWS($A$1:A19)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
+        <v>Week 4: 25 Jan-29 Jan</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C27" t="s">
-        <v>23</v>
-      </c>
-      <c r="D27" s="4" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A28" s="3" t="str">
-        <f ca="1">"Week "&amp;_xlfn.LET(_xlpm.d,TODAY()+7*(ROWS($A$1:A22)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
+        <f>"Week "&amp;_xlfn.LET(_xlpm.d,"21-9-2026"+7*(ROWS($A$1:A20)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
+        <v>Week 5: 1 Feb-5 Feb</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C28" t="s">
+        <v>30</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A29" s="17" t="str">
+        <f>"Week "&amp;_xlfn.LET(_xlpm.d,"21-9-2026"+7*(ROWS($A$1:A21)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
+        <v>Week 6: 8 Feb-12 Feb</v>
+      </c>
+      <c r="B29" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="D29" s="9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A30" s="3" t="str">
+        <f>"Week "&amp;_xlfn.LET(_xlpm.d,"21-9-2026"+7*(ROWS($A$1:A22)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
         <v>Week 7: 15 Feb-19 Feb</v>
       </c>
-      <c r="B28" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="C28" t="s">
-        <v>21</v>
-      </c>
-      <c r="D28" s="4" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="A29" s="3" t="str">
-        <f ca="1">"Week "&amp;_xlfn.LET(_xlpm.d,TODAY()+7*(ROWS($A$1:A23)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
+      <c r="B30" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C30" t="s">
+        <v>18</v>
+      </c>
+      <c r="D30" s="17"/>
+    </row>
+    <row r="31" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A31" s="3" t="str">
+        <f>"Week "&amp;_xlfn.LET(_xlpm.d,"21-9-2026"+7*(ROWS($A$1:A23)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
         <v>Week 8: 22 Feb-26 Feb</v>
       </c>
-      <c r="B29" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="C29" t="s">
-        <v>21</v>
-      </c>
-      <c r="D29" s="4"/>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A30" s="11" t="str">
-        <f ca="1">"Week "&amp;_xlfn.LET(_xlpm.d,TODAY()+7*(ROWS($A$1:A24)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
+      <c r="B31" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C31" t="s">
+        <v>18</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A32" s="3" t="str">
+        <f>"Week "&amp;_xlfn.LET(_xlpm.d,"21-9-2026"+7*(ROWS($A$1:A24)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
         <v>Week 9: 1 Mar-5 Mar</v>
       </c>
-      <c r="B30" s="12"/>
-      <c r="C30" s="13"/>
-      <c r="D30" s="13"/>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A31" s="9" t="str">
-        <f ca="1">"Week "&amp;_xlfn.LET(_xlpm.d,TODAY()+7*(ROWS($A$1:A25)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
+      <c r="B32" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C32" t="s">
+        <v>18</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A33" s="3" t="str">
+        <f>"Week "&amp;_xlfn.LET(_xlpm.d,"21-9-2026"+7*(ROWS($A$1:A25)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
         <v>Week 10: 8 Mar-12 Mar</v>
       </c>
-      <c r="B31" s="10"/>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A32" s="9" t="str">
-        <f ca="1">"Week "&amp;_xlfn.LET(_xlpm.d,TODAY()+7*(ROWS($A$1:A26)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
+      <c r="B33" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C33" t="s">
+        <v>16</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A34" s="2" t="str">
+        <f>"Week "&amp;_xlfn.LET(_xlpm.d,"21-9-2026"+7*(ROWS($A$1:A26)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
         <v>Week 11: 15 Mar-19 Mar</v>
       </c>
-      <c r="B32" s="10"/>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A33" s="9" t="str">
-        <f ca="1">"Week "&amp;_xlfn.LET(_xlpm.d,TODAY()+7*(ROWS($A$1:A27)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
+      <c r="B34" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D34" s="19" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A35" s="3" t="str">
+        <f>"Week "&amp;_xlfn.LET(_xlpm.d,"21-9-2026"+7*(ROWS($A$1:A27)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
         <v>Week 12: 22 Mar-26 Mar</v>
       </c>
-      <c r="B33" s="10"/>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A34" s="9" t="str">
-        <f ca="1">"Week "&amp;_xlfn.LET(_xlpm.d,TODAY()+7*(ROWS($A$1:A28)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
+      <c r="B35" s="8"/>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A36" s="3" t="str">
+        <f>"Week "&amp;_xlfn.LET(_xlpm.d,"21-9-2026"+7*(ROWS($A$1:A28)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
         <v>Week 13: 29 Mar-2 Apr</v>
       </c>
-      <c r="B34" s="10"/>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A35" s="9" t="str">
-        <f ca="1">"Week "&amp;_xlfn.LET(_xlpm.d,TODAY()+7*(ROWS($A$1:A29)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
+      <c r="B36" s="8"/>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A37" s="3" t="str">
+        <f>"Week "&amp;_xlfn.LET(_xlpm.d,"21-9-2026"+7*(ROWS($A$1:A29)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
         <v>Week 14: 5 Apr-9 Apr</v>
       </c>
-      <c r="B35" s="10"/>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A36" s="9" t="str">
-        <f ca="1">"Week "&amp;_xlfn.LET(_xlpm.d,TODAY()+7*(ROWS($A$1:A30)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
+      <c r="B37" s="8"/>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A38" s="3" t="str">
+        <f>"Week "&amp;_xlfn.LET(_xlpm.d,"21-9-2026"+7*(ROWS($A$1:A30)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
         <v>Week 15: 12 Apr-16 Apr</v>
       </c>
-      <c r="B36" s="10"/>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A37" s="9" t="str">
-        <f ca="1">"Week "&amp;_xlfn.LET(_xlpm.d,TODAY()+7*(ROWS($A$1:A31)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
+      <c r="B38" s="8"/>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A39" s="3" t="str">
+        <f>"Week "&amp;_xlfn.LET(_xlpm.d,"21-9-2026"+7*(ROWS($A$1:A31)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
         <v>Week 16: 19 Apr-23 Apr</v>
       </c>
-      <c r="B37" s="10"/>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A38" s="9" t="str">
-        <f ca="1">"Week "&amp;_xlfn.LET(_xlpm.d,TODAY()+7*(ROWS($A$1:A32)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
-        <v>Week 17: 26 Apr-30 Apr</v>
-      </c>
-      <c r="B38" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added new papers to Docs map
</commit_message>
<xml_diff>
--- a/Docs/Thesis planning.xlsx
+++ b/Docs/Thesis planning.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/LaptopvanFrank/Desktop/Cardano/Thesis/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/LaptopvanFrank/Desktop/Cardano/Thesis/Fulcrum/Docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{286A0EFA-9132-8348-9033-45B65205F6B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A26AB4CB-0226-964A-8EEE-4A347A53D400}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="34560" windowHeight="21600" xr2:uid="{C4A47A45-E97D-B144-962D-ED697A072EEA}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20460" xr2:uid="{C4A47A45-E97D-B144-962D-ED697A072EEA}"/>
   </bookViews>
   <sheets>
     <sheet name="-" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="45">
   <si>
     <t xml:space="preserve">Thesis planning </t>
   </si>
@@ -136,9 +136,6 @@
     <t>Resultaten + Verslag</t>
   </si>
   <si>
-    <t>Probleemomschrijving + Model Formulation Final</t>
-  </si>
-  <si>
     <t>Probleemomschrijving + Model Formulation Proposal</t>
   </si>
   <si>
@@ -172,6 +169,15 @@
   </si>
   <si>
     <t>Base case model script + progressie PP</t>
+  </si>
+  <si>
+    <t>Model Formulation Final</t>
+  </si>
+  <si>
+    <t>Probleemomschrijving</t>
+  </si>
+  <si>
+    <t>1. LDI Staatsobligaties kwartaalupdate Achmea IM Q3</t>
   </si>
 </sst>
 </file>
@@ -408,7 +414,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -430,7 +436,6 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="7" xfId="3" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1060,15 +1065,18 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B3" t="s">
         <v>17</v>
+      </c>
+      <c r="D3" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
@@ -1110,54 +1118,54 @@
       </c>
     </row>
     <row r="9" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A9" s="21" t="str">
+      <c r="A9" s="20" t="str">
         <f>"Week "&amp;_xlfn.LET(_xlpm.d,"21-9-2026"+7*(ROWS($A$1:A1)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
         <v>Week 39: 21 Sep-25 Sep</v>
       </c>
-      <c r="B9" s="22" t="s">
+      <c r="B9" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="23" t="s">
+      <c r="C9" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="24" t="s">
+      <c r="D9" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="F9" s="26" t="s">
-        <v>37</v>
+      <c r="F9" s="25" t="s">
+        <v>36</v>
       </c>
       <c r="G9" s="12"/>
     </row>
     <row r="10" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A10" s="21" t="str">
+      <c r="A10" s="20" t="str">
         <f>"Week "&amp;_xlfn.LET(_xlpm.d,"21-9-2026"+7*(ROWS($A$1:A2)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
         <v>Week 40: 28 Sep-2 Oct</v>
       </c>
-      <c r="B10" s="22" t="s">
+      <c r="B10" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="23" t="s">
+      <c r="C10" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="D10" s="25"/>
+      <c r="D10" s="24"/>
       <c r="F10" s="13" t="s">
         <v>11</v>
       </c>
       <c r="G10" s="14"/>
     </row>
     <row r="11" spans="1:7" ht="35" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="21" t="str">
+      <c r="A11" s="20" t="str">
         <f>"Week "&amp;_xlfn.LET(_xlpm.d,"21-9-2026"+7*(ROWS($A$1:A3)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
         <v>Week 41: 5 Oct-9 Oct</v>
       </c>
-      <c r="B11" s="22" t="s">
+      <c r="B11" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="23" t="s">
+      <c r="C11" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="D11" s="24" t="s">
-        <v>32</v>
+      <c r="D11" s="23" t="s">
+        <v>31</v>
       </c>
       <c r="F11" s="15" t="s">
         <v>12</v>
@@ -1165,31 +1173,31 @@
       <c r="G11" s="16"/>
     </row>
     <row r="12" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A12" s="21" t="str">
+      <c r="A12" s="20" t="str">
         <f>"Week "&amp;_xlfn.LET(_xlpm.d,"21-9-2026"+7*(ROWS($A$1:A4)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
         <v>Week 42: 12 Oct-16 Oct</v>
       </c>
-      <c r="B12" s="22" t="s">
+      <c r="B12" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="C12" s="23" t="s">
+      <c r="C12" s="22" t="s">
         <v>14</v>
       </c>
       <c r="D12" s="4"/>
     </row>
     <row r="13" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A13" s="3" t="str">
+      <c r="A13" s="20" t="str">
         <f>"Week "&amp;_xlfn.LET(_xlpm.d,"21-9-2026"+7*(ROWS($A$1:A5)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
         <v>Week 43: 19 Oct-23 Oct</v>
       </c>
-      <c r="B13" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="C13" t="s">
+      <c r="B13" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" s="22" t="s">
+        <v>40</v>
+      </c>
+      <c r="D13" s="23" t="s">
         <v>41</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>42</v>
       </c>
       <c r="F13" s="7"/>
     </row>
@@ -1205,7 +1213,7 @@
         <v>26</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>31</v>
+        <v>43</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="34" x14ac:dyDescent="0.2">
@@ -1219,7 +1227,9 @@
       <c r="C15" t="s">
         <v>26</v>
       </c>
-      <c r="D15" s="4"/>
+      <c r="D15" s="4" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="16" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="str">
@@ -1232,9 +1242,6 @@
       <c r="C16" t="s">
         <v>26</v>
       </c>
-      <c r="D16" s="4" t="s">
-        <v>25</v>
-      </c>
     </row>
     <row r="17" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="str">
@@ -1247,7 +1254,9 @@
       <c r="C17" t="s">
         <v>27</v>
       </c>
-      <c r="D17" s="4"/>
+      <c r="D17" s="4" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="18" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A18" s="3" t="str">
@@ -1321,7 +1330,7 @@
         <v>Week 53: 28 Dec-1 Jan</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C23" s="6" t="s">
         <v>19</v>
@@ -1354,7 +1363,7 @@
         <v>27</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="34" x14ac:dyDescent="0.2">
@@ -1397,15 +1406,15 @@
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A29" s="17" t="str">
+      <c r="A29" t="str">
         <f>"Week "&amp;_xlfn.LET(_xlpm.d,"21-9-2026"+7*(ROWS($A$1:A21)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
         <v>Week 6: 8 Feb-12 Feb</v>
       </c>
-      <c r="B29" s="20" t="s">
-        <v>35</v>
+      <c r="B29" s="19" t="s">
+        <v>34</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D29" s="9" t="s">
         <v>20</v>
@@ -1422,7 +1431,6 @@
       <c r="C30" t="s">
         <v>18</v>
       </c>
-      <c r="D30" s="17"/>
     </row>
     <row r="31" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A31" s="3" t="str">
@@ -1474,14 +1482,14 @@
         <f>"Week "&amp;_xlfn.LET(_xlpm.d,"21-9-2026"+7*(ROWS($A$1:A26)-1),_xlfn.ISOWEEKNUM(_xlpm.d)&amp;": "&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+1,"d mmm")&amp;"-"&amp;TEXT(_xlpm.d-WEEKDAY(_xlpm.d,2)+5,"d mmm"))</f>
         <v>Week 11: 15 Mar-19 Mar</v>
       </c>
-      <c r="B34" s="18" t="s">
+      <c r="B34" s="17" t="s">
         <v>21</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D34" s="19" t="s">
-        <v>33</v>
+      <c r="D34" s="18" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
@@ -1520,6 +1528,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>